<commit_message>
Update Beacon Peak (滶蕴) unsold units to include 5% base discount and 120-day 6% early settlement cash rebate popup calculation
</commit_message>
<xml_diff>
--- a/files/九龙-石硖尾-滶蕴.xlsx
+++ b/files/九龙-石硖尾-滶蕴.xlsx
@@ -1074,7 +1074,7 @@
       </c>
       <c r="M7" s="3" t="inlineStr">
         <is>
-          <t>建築期備⽤⼀按貸款付款計劃</t>
+          <t>現金付款計劃 (減5%) + 120天提前成交現金回贈6%</t>
         </is>
       </c>
       <c r="N7" s="3" t="inlineStr">
@@ -1206,7 +1206,7 @@
       </c>
       <c r="M9" s="3" t="inlineStr">
         <is>
-          <t>建築期備⽤⼀按貸款付款計劃</t>
+          <t>現金付款計劃 (減5%) + 120天提前成交現金回贈6%</t>
         </is>
       </c>
       <c r="N9" s="3" t="inlineStr">
@@ -1268,7 +1268,7 @@
       </c>
       <c r="M10" s="3" t="inlineStr">
         <is>
-          <t>建築期備⽤⼀按貸款付款計劃</t>
+          <t>現金付款計劃 (減5%) + 120天提前成交現金回贈6%</t>
         </is>
       </c>
       <c r="N10" s="3" t="inlineStr">
@@ -1330,7 +1330,7 @@
       </c>
       <c r="M11" s="3" t="inlineStr">
         <is>
-          <t>建築期備⽤⼀按貸款付款計劃</t>
+          <t>現金付款計劃 (減5%) + 120天提前成交現金回贈6%</t>
         </is>
       </c>
       <c r="N11" s="3" t="inlineStr">
@@ -1392,7 +1392,7 @@
       </c>
       <c r="M12" s="3" t="inlineStr">
         <is>
-          <t>建築期備⽤⼀按貸款付款計劃</t>
+          <t>現金付款計劃 (減5%) + 120天提前成交現金回贈6%</t>
         </is>
       </c>
       <c r="N12" s="3" t="inlineStr">
@@ -1454,7 +1454,7 @@
       </c>
       <c r="M13" s="3" t="inlineStr">
         <is>
-          <t>建築期備⽤⼀按貸款付款計劃</t>
+          <t>現金付款計劃 (減5%) + 120天提前成交現金回贈6%</t>
         </is>
       </c>
       <c r="N13" s="3" t="inlineStr">
@@ -1516,7 +1516,7 @@
       </c>
       <c r="M14" s="3" t="inlineStr">
         <is>
-          <t>建築期備⽤⼀按貸款付款計劃</t>
+          <t>現金付款計劃 (減5%) + 120天提前成交現金回贈6%</t>
         </is>
       </c>
       <c r="N14" s="3" t="inlineStr">
@@ -2168,7 +2168,7 @@
       </c>
       <c r="M24" s="3" t="inlineStr">
         <is>
-          <t>建築期備⽤⼀按貸款付款計劃</t>
+          <t>現金付款計劃 (減5%) + 120天提前成交現金回贈6%</t>
         </is>
       </c>
       <c r="N24" s="3" t="inlineStr">
@@ -2230,7 +2230,7 @@
       </c>
       <c r="M25" s="3" t="inlineStr">
         <is>
-          <t>建築期備⽤⼀按貸款付款計劃</t>
+          <t>現金付款計劃 (減5%) + 120天提前成交現金回贈6%</t>
         </is>
       </c>
       <c r="N25" s="3" t="inlineStr">
@@ -2292,7 +2292,7 @@
       </c>
       <c r="M26" s="3" t="inlineStr">
         <is>
-          <t>建築期備⽤⼀按貸款付款計劃</t>
+          <t>現金付款計劃 (減5%) + 120天提前成交現金回贈6%</t>
         </is>
       </c>
       <c r="N26" s="3" t="inlineStr">
@@ -2416,7 +2416,7 @@
       </c>
       <c r="M28" s="3" t="inlineStr">
         <is>
-          <t>建築期備⽤⼀按貸款付款計劃</t>
+          <t>現金付款計劃 (減5%) + 120天提前成交現金回贈6%</t>
         </is>
       </c>
       <c r="N28" s="3" t="inlineStr">
@@ -3308,7 +3308,7 @@
       </c>
       <c r="M42" s="3" t="inlineStr">
         <is>
-          <t>建築期備⽤⼀按貸款付款計劃</t>
+          <t>現金付款計劃 (減5%) + 120天提前成交現金回贈6%</t>
         </is>
       </c>
       <c r="N42" s="3" t="inlineStr">
@@ -3370,7 +3370,7 @@
       </c>
       <c r="M43" s="3" t="inlineStr">
         <is>
-          <t>建築期備⽤⼀按貸款付款計劃</t>
+          <t>現金付款計劃 (減5%) + 120天提前成交現金回贈6%</t>
         </is>
       </c>
       <c r="N43" s="3" t="inlineStr">
@@ -3432,7 +3432,7 @@
       </c>
       <c r="M44" s="3" t="inlineStr">
         <is>
-          <t>建築期備⽤⼀按貸款付款計劃</t>
+          <t>現金付款計劃 (減5%) + 120天提前成交現金回贈6%</t>
         </is>
       </c>
       <c r="N44" s="3" t="inlineStr">
@@ -3556,7 +3556,7 @@
       </c>
       <c r="M46" s="3" t="inlineStr">
         <is>
-          <t>建築期備⽤⼀按貸款付款計劃</t>
+          <t>現金付款計劃 (減5%) + 120天提前成交現金回贈6%</t>
         </is>
       </c>
       <c r="N46" s="3" t="inlineStr">
@@ -4200,7 +4200,7 @@
       </c>
       <c r="M56" s="3" t="inlineStr">
         <is>
-          <t>建築期備⽤⼀按貸款付款計劃</t>
+          <t>現金付款計劃 (減5%) + 120天提前成交現金回贈6%</t>
         </is>
       </c>
       <c r="N56" s="3" t="inlineStr">
@@ -4262,7 +4262,7 @@
       </c>
       <c r="M57" s="3" t="inlineStr">
         <is>
-          <t>建築期備⽤⼀按貸款付款計劃</t>
+          <t>現金付款計劃 (減5%) + 120天提前成交現金回贈6%</t>
         </is>
       </c>
       <c r="N57" s="3" t="inlineStr">
@@ -5332,7 +5332,7 @@
       </c>
       <c r="M74" s="3" t="inlineStr">
         <is>
-          <t>建築期備⽤⼀按貸款付款計劃</t>
+          <t>現金付款計劃 (減5%) + 120天提前成交現金回贈6%</t>
         </is>
       </c>
       <c r="N74" s="3" t="inlineStr">
@@ -5580,7 +5580,7 @@
       </c>
       <c r="M78" s="3" t="inlineStr">
         <is>
-          <t>建築期備⽤⼀按貸款付款計劃</t>
+          <t>現金付款計劃 (減5%) + 120天提前成交現金回贈6%</t>
         </is>
       </c>
       <c r="N78" s="3" t="inlineStr">
@@ -6224,7 +6224,7 @@
       </c>
       <c r="M88" s="3" t="inlineStr">
         <is>
-          <t>建築期備⽤⼀按貸款付款計劃</t>
+          <t>現金付款計劃 (減5%) + 120天提前成交現金回贈6%</t>
         </is>
       </c>
       <c r="N88" s="3" t="inlineStr">
@@ -6286,7 +6286,7 @@
       </c>
       <c r="M89" s="3" t="inlineStr">
         <is>
-          <t>建築期備⽤⼀按貸款付款計劃</t>
+          <t>現金付款計劃 (減5%) + 120天提前成交現金回贈6%</t>
         </is>
       </c>
       <c r="N89" s="3" t="inlineStr">
@@ -6348,7 +6348,7 @@
       </c>
       <c r="M90" s="3" t="inlineStr">
         <is>
-          <t>建築期備⽤⼀按貸款付款計劃</t>
+          <t>現金付款計劃 (減5%) + 120天提前成交現金回贈6%</t>
         </is>
       </c>
       <c r="N90" s="3" t="inlineStr">
@@ -6472,7 +6472,7 @@
       </c>
       <c r="M92" s="3" t="inlineStr">
         <is>
-          <t>建築期備⽤⼀按貸款付款計劃</t>
+          <t>現金付款計劃 (減5%) + 120天提前成交現金回贈6%</t>
         </is>
       </c>
       <c r="N92" s="3" t="inlineStr">

</xml_diff>